<commit_message>
Fix empty MSX and USA upload templates.
Use a single visible Holdings sheet and serve templates through an API route so downloads open with headers, instructions, and sample rows in Excel.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/msx-upload-template.xlsx
+++ b/public/templates/msx-upload-template.xlsx
@@ -4,7 +4,6 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Holdings" sheetId="1" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K10"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -415,200 +414,75 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Symbol</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Quantity</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Cost Basis</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Market Price</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Market Value</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Unrealised P&amp;L</v>
-      </c>
-      <c r="H1" t="str">
-        <v>ISIN</v>
-      </c>
-      <c r="I1" t="str">
-        <v>CUSIP</v>
-      </c>
-      <c r="J1" t="str">
-        <v>SEDOL</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Exchange</v>
+        <v>MSX Brokerage Upload Template</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BKMB</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Bank Muscat SAOG</v>
-      </c>
-      <c r="C2">
-        <v>5000</v>
-      </c>
-      <c r="D2">
-        <v>4250</v>
-      </c>
-      <c r="E2">
-        <v>0.92</v>
-      </c>
-      <c r="F2">
-        <v>4600</v>
-      </c>
-      <c r="G2">
-        <v>350</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v>MSX</v>
+        <v>Fill in your holdings below. Symbol and Quantity are required. Delete the sample rows or replace them.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>OQGN</v>
-      </c>
-      <c r="B3" t="str">
-        <v>OQ Exploration &amp; Production</v>
-      </c>
-      <c r="C3">
-        <v>10000</v>
-      </c>
-      <c r="D3">
-        <v>1200</v>
-      </c>
-      <c r="E3">
-        <v>0.135</v>
-      </c>
-      <c r="F3">
-        <v>1350</v>
-      </c>
-      <c r="G3">
-        <v>150</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <v>MSX</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>GULF</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Gulf Investment House</v>
-      </c>
-      <c r="C4">
-        <v>2500</v>
-      </c>
-      <c r="D4">
-        <v>187.5</v>
-      </c>
-      <c r="E4">
-        <v>0.082</v>
-      </c>
-      <c r="F4">
-        <v>205</v>
-      </c>
-      <c r="G4">
-        <v>17.5</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4" t="str">
-        <v>MSX</v>
+        <v>Symbol format: 2-6 letter codes (e.g. BKMB, OQGN). Amounts are in OMR.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>NBOB</v>
+        <v>Symbol</v>
       </c>
       <c r="B5" t="str">
-        <v>National Bank of Oman</v>
-      </c>
-      <c r="C5">
-        <v>3000</v>
-      </c>
-      <c r="D5">
-        <v>900</v>
-      </c>
-      <c r="E5">
-        <v>0.315</v>
-      </c>
-      <c r="F5">
-        <v>945</v>
-      </c>
-      <c r="G5">
-        <v>45</v>
+        <v>Name</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Quantity</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Cost Basis</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Market Price</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Market Value</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Unrealised P&amp;L</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>ISIN</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>CUSIP</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>SEDOL</v>
       </c>
       <c r="K5" t="str">
-        <v>MSX</v>
+        <v>Exchange</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ZAIN</v>
+        <v>BKMB</v>
       </c>
       <c r="B6" t="str">
-        <v>Oman Telecommunications</v>
+        <v>Bank Muscat SAOG</v>
       </c>
       <c r="C6">
-        <v>8000</v>
+        <v>5000</v>
       </c>
       <c r="D6">
-        <v>640</v>
+        <v>4250</v>
       </c>
       <c r="E6">
-        <v>0.085</v>
+        <v>0.92</v>
       </c>
       <c r="F6">
-        <v>680</v>
+        <v>4600</v>
       </c>
       <c r="G6">
-        <v>40</v>
+        <v>350</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -623,181 +497,149 @@
         <v>MSX</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>OQGN</v>
+      </c>
+      <c r="B7" t="str">
+        <v>OQ Exploration &amp; Production</v>
+      </c>
+      <c r="C7">
+        <v>10000</v>
+      </c>
+      <c r="D7">
+        <v>1200</v>
+      </c>
+      <c r="E7">
+        <v>0.135</v>
+      </c>
+      <c r="F7">
+        <v>1350</v>
+      </c>
+      <c r="G7">
+        <v>150</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>MSX</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>GULF</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Gulf Investment House</v>
+      </c>
+      <c r="C8">
+        <v>2500</v>
+      </c>
+      <c r="D8">
+        <v>187.5</v>
+      </c>
+      <c r="E8">
+        <v>0.082</v>
+      </c>
+      <c r="F8">
+        <v>205</v>
+      </c>
+      <c r="G8">
+        <v>17.5</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>MSX</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>NBOB</v>
+      </c>
+      <c r="B9" t="str">
+        <v>National Bank of Oman</v>
+      </c>
+      <c r="C9">
+        <v>3000</v>
+      </c>
+      <c r="D9">
+        <v>900</v>
+      </c>
+      <c r="E9">
+        <v>0.315</v>
+      </c>
+      <c r="F9">
+        <v>945</v>
+      </c>
+      <c r="G9">
+        <v>45</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>MSX</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ZAIN</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Oman Telecommunications</v>
+      </c>
+      <c r="C10">
+        <v>8000</v>
+      </c>
+      <c r="D10">
+        <v>640</v>
+      </c>
+      <c r="E10">
+        <v>0.085</v>
+      </c>
+      <c r="F10">
+        <v>680</v>
+      </c>
+      <c r="G10">
+        <v>40</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>MSX</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B26"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="72.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>MSX — Brokerage Upload Template</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>How to use</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>1. Fill the Holdings sheet with your positions (Symbol and Quantity are required).</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2. Save as .xlsx and upload via Portfolio → MSX → Import Brokerage Reports.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>3. Select the entity that owns these holdings before uploading.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Column guide</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Symbol</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ticker code — 2–6 letter codes (e.g. BKMB, OQGN)</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Name</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Security name (optional)</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Quantity</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Number of shares/units held (required)</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Cost Basis</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Total purchase cost for the position (OMR)</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Market Price</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Latest price per share (OMR)</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Market Value</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Current position value (OMR)</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Unrealised P&amp;L</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Gain or loss vs cost basis</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>ISIN / CUSIP / SEDOL</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Security identifiers when available</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Exchange</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Listing exchange (optional; defaults to NYSE/NASDAQ for USA)</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Accepted file formats</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>PDF and Excel (.xlsx, .xls)</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>• Delete the sample rows before uploading your real portfolio, or replace them.</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>• Broker exports with different column names (Ticker, Shares, LTP, etc.) are also supported.</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>• MSX accepts PDF and Excel; you can also upload native broker statements directly.</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>• Closing prices sync automatically from msx.om after market close (Sun–Thu).</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix blank Excel exports by switching to ExcelJS.
Generate upload templates and holdings exports with ExcelJS and serve template downloads through server actions so files open correctly in Microsoft Excel.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/msx-upload-template.xlsx
+++ b/public/templates/msx-upload-template.xlsx
@@ -1,47 +1,107 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Holdings" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Holdings" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
+  <si>
+    <t>MSX Brokerage Upload Template</t>
+  </si>
+  <si>
+    <t>Fill in your holdings below. Symbol and Quantity are required. Delete the sample rows or replace them.</t>
+  </si>
+  <si>
+    <t>Symbol format: 2-6 letter codes (e.g. BKMB, OQGN). Amounts are in OMR.</t>
+  </si>
+  <si>
+    <t>Symbol</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Cost Basis</t>
+  </si>
+  <si>
+    <t>Market Price</t>
+  </si>
+  <si>
+    <t>Market Value</t>
+  </si>
+  <si>
+    <t>Unrealised P&amp;L</t>
+  </si>
+  <si>
+    <t>ISIN</t>
+  </si>
+  <si>
+    <t>CUSIP</t>
+  </si>
+  <si>
+    <t>SEDOL</t>
+  </si>
+  <si>
+    <t>Exchange</t>
+  </si>
+  <si>
+    <t>BKMB</t>
+  </si>
+  <si>
+    <t>Bank Muscat SAOG</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>MSX</t>
+  </si>
+  <si>
+    <t>OQGN</t>
+  </si>
+  <si>
+    <t>OQ Exploration &amp; Production</t>
+  </si>
+  <si>
+    <t>GULF</t>
+  </si>
+  <si>
+    <t>Gulf Investment House</t>
+  </si>
+  <si>
+    <t>NBOB</t>
+  </si>
+  <si>
+    <t>National Bank of Oman</t>
+  </si>
+  <si>
+    <t>ZAIN</t>
+  </si>
+  <si>
+    <t>Oman Telecommunications</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,13 +125,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,78 +464,66 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K10"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>MSX Brokerage Upload Template</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Fill in your holdings below. Symbol and Quantity are required. Delete the sample rows or replace them.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Symbol format: 2-6 letter codes (e.g. BKMB, OQGN). Amounts are in OMR.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Symbol</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Name</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Quantity</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Cost Basis</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Market Price</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Market Value</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Unrealised P&amp;L</v>
-      </c>
-      <c r="H5" t="str">
-        <v>ISIN</v>
-      </c>
-      <c r="I5" t="str">
-        <v>CUSIP</v>
-      </c>
-      <c r="J5" t="str">
-        <v>SEDOL</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Exchange</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>BKMB</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Bank Muscat SAOG</v>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
       </c>
       <c r="C6">
         <v>5000</v>
@@ -484,25 +540,25 @@
       <c r="G6">
         <v>350</v>
       </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" t="str">
-        <v>MSX</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>OQGN</v>
-      </c>
-      <c r="B7" t="str">
-        <v>OQ Exploration &amp; Production</v>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
       </c>
       <c r="C7">
         <v>10000</v>
@@ -519,25 +575,25 @@
       <c r="G7">
         <v>150</v>
       </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v>MSX</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>GULF</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Gulf Investment House</v>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
       </c>
       <c r="C8">
         <v>2500</v>
@@ -554,25 +610,25 @@
       <c r="G8">
         <v>17.5</v>
       </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <v/>
-      </c>
-      <c r="K8" t="str">
-        <v>MSX</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>NBOB</v>
-      </c>
-      <c r="B9" t="str">
-        <v>National Bank of Oman</v>
+      <c r="H8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
       </c>
       <c r="C9">
         <v>3000</v>
@@ -589,25 +645,25 @@
       <c r="G9">
         <v>45</v>
       </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v/>
-      </c>
-      <c r="K9" t="str">
-        <v>MSX</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>ZAIN</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Oman Telecommunications</v>
+      <c r="H9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" t="s">
+        <v>16</v>
+      </c>
+      <c r="K9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
       </c>
       <c r="C10">
         <v>8000</v>
@@ -624,22 +680,21 @@
       <c r="G10">
         <v>40</v>
       </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <v/>
-      </c>
-      <c r="K10" t="str">
-        <v>MSX</v>
+      <c r="H10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" t="s">
+        <v>16</v>
+      </c>
+      <c r="K10" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K10"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>